<commit_message>
Updated lab 5 and 8 rubrics
</commit_message>
<xml_diff>
--- a/Labs/Lab05/CS133JS_Lab05_Rubric.xlsx
+++ b/Labs/Lab05/CS133JS_Lab05_Rubric.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repos\CS133JS-CourseMaterials\Labs\Lab05\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repos\CS133JS-Repos\CS133JS-CourseMaterials\Labs\Lab05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70E55AA5-4468-4055-9287-BFF66E5F811C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{288CB742-1270-4CC3-8694-D1A8C3C96537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="4092" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{9702CE45-50CE-F14F-802C-E5FE921247A2}"/>
+    <workbookView xWindow="30708" yWindow="4236" windowWidth="16728" windowHeight="12960" activeTab="1" xr2:uid="{9702CE45-50CE-F14F-802C-E5FE921247A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Rubric" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="26">
   <si>
     <t>Criteria</t>
   </si>
@@ -57,12 +57,6 @@
     <t>Part 2</t>
   </si>
   <si>
-    <t>Developer’s name, date in comments in each file</t>
-  </si>
-  <si>
-    <t>Review of your code with completed "Prod." column</t>
-  </si>
-  <si>
     <t>Web app 1 functionality</t>
   </si>
   <si>
@@ -109,6 +103,18 @@
   </si>
   <si>
     <t>Here's the grade breakdown:</t>
+  </si>
+  <si>
+    <t>No errors (syntax, console or crash)</t>
+  </si>
+  <si>
+    <t>No console errors</t>
+  </si>
+  <si>
+    <t>"use strict" added to .js files</t>
+  </si>
+  <si>
+    <t>Both web apps:</t>
   </si>
 </sst>
 </file>
@@ -165,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -179,6 +185,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -493,22 +500,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3216228F-B421-8943-9C69-C9FAC1E7C520}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="2.69921875" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="6" max="6" width="1.296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -530,63 +536,50 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E6">
         <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3"/>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9">
-        <v>3</v>
+      <c r="A9" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="B10" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E10">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="B11" t="s">
-        <v>14</v>
-      </c>
+      <c r="B11" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="7"/>
       <c r="E11">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12">
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="B13" t="s">
-        <v>15</v>
       </c>
       <c r="E13">
         <v>3</v>
@@ -594,51 +587,99 @@
     </row>
     <row r="14" spans="1:5">
       <c r="B14" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E14">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" t="s">
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="B16" t="s">
         <v>12</v>
       </c>
-      <c r="E15">
+      <c r="E16">
         <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" t="s">
-        <v>7</v>
-      </c>
-      <c r="E16">
-        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="B19" t="s">
+        <v>22</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="B20" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20">
         <v>3</v>
       </c>
-      <c r="E18">
-        <f>SUM(E6:E16)</f>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="B21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="E23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E25">
+        <f>SUM(E6:E23)</f>
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
-      <c r="A20">
-        <v>1</v>
-      </c>
-      <c r="B20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22">
+    <row r="27" spans="1:5">
+      <c r="A27">
+        <v>1</v>
+      </c>
+      <c r="B27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29">
         <v>2</v>
       </c>
-      <c r="B22" t="s">
-        <v>16</v>
+      <c r="B29" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -649,11 +690,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5839EC90-C7F0-3A4B-8678-BE197ECC720E}">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="7" customWidth="1"/>
-    <col min="4" max="4" width="4.796875" customWidth="1"/>
+    <col min="1" max="1" width="3.796875" customWidth="1"/>
+    <col min="4" max="4" width="7.296875" customWidth="1"/>
     <col min="5" max="5" width="8" customWidth="1"/>
     <col min="6" max="6" width="5.69921875" customWidth="1"/>
     <col min="7" max="7" width="1.296875" customWidth="1"/>
@@ -662,17 +703,17 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -684,7 +725,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -705,7 +746,7 @@
         <v>2</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -718,7 +759,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E7">
         <v>8</v>
@@ -736,7 +777,7 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -747,132 +788,170 @@
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
+      <c r="A10" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
       <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="H10" s="4"/>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11">
         <v>3</v>
       </c>
-      <c r="F10">
+      <c r="F11">
         <v>3</v>
-      </c>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="B11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11">
-        <v>2</v>
-      </c>
-      <c r="F11">
-        <v>2</v>
       </c>
       <c r="H11" s="4"/>
     </row>
     <row r="12" spans="1:8">
       <c r="B12" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E12">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F12">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H12" s="4"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" t="s">
-        <v>9</v>
+      <c r="B13" t="s">
+        <v>11</v>
       </c>
       <c r="E13">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F13">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H13" s="4"/>
     </row>
     <row r="14" spans="1:8">
       <c r="B14" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E14">
+        <v>4</v>
+      </c>
+      <c r="F14">
+        <v>4</v>
+      </c>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15">
+        <v>5</v>
+      </c>
+      <c r="F15">
+        <v>5</v>
+      </c>
+      <c r="H15" s="4"/>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="B16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="H16" s="4"/>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="B17" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17">
         <v>3</v>
       </c>
-      <c r="F14">
+      <c r="F17">
         <v>3</v>
       </c>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="B15" t="s">
-        <v>14</v>
-      </c>
-      <c r="E15">
-        <v>6</v>
-      </c>
-      <c r="F15">
-        <v>6</v>
-      </c>
-      <c r="H15" s="4"/>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" t="s">
+      <c r="H17" s="4"/>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="B18" t="s">
         <v>12</v>
       </c>
-      <c r="E16">
-        <v>4</v>
-      </c>
-      <c r="F16">
-        <v>4</v>
-      </c>
-      <c r="H16" s="4"/>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17">
-        <v>2</v>
-      </c>
-      <c r="F17">
-        <v>2</v>
-      </c>
-      <c r="H17" s="4"/>
-    </row>
-    <row r="18" spans="1:8">
+      <c r="E18">
+        <v>5</v>
+      </c>
+      <c r="F18">
+        <v>5</v>
+      </c>
       <c r="H18" s="4"/>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19">
+        <v>4</v>
+      </c>
+      <c r="F19">
+        <v>4</v>
+      </c>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" t="s">
+        <v>17</v>
+      </c>
+      <c r="E20">
+        <v>2</v>
+      </c>
+      <c r="F20">
+        <v>2</v>
+      </c>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
         <v>3</v>
       </c>
-      <c r="E19">
-        <f>SUM(E7:E17)</f>
+      <c r="E22">
+        <f>SUM(E7:E20)</f>
         <v>40</v>
       </c>
-      <c r="F19">
-        <f>SUM(F7:F17)</f>
+      <c r="F22">
+        <f>SUM(F7:F20)</f>
         <v>40</v>
       </c>
-      <c r="H19" s="4"/>
-    </row>
-    <row r="21" spans="1:8">
-      <c r="A21">
-        <v>1</v>
-      </c>
-      <c r="B21" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23">
+      <c r="H22" s="4"/>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24">
+        <v>1</v>
+      </c>
+      <c r="B24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26">
         <v>2</v>
       </c>
-      <c r="B23" t="s">
-        <v>16</v>
+      <c r="B26" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>